<commit_message>
Update game flow config data
</commit_message>
<xml_diff>
--- a/Config/Luban/Datas/#game.buff.xlsx
+++ b/Config/Luban/Datas/#game.buff.xlsx
@@ -510,12 +510,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="5"/>
-    <col width="14" customWidth="1" min="6" max="15"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="5"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="15"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -541,22 +545,17 @@
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>type</t>
+          <t>effects#format=json</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>effects#format=json</t>
+          <t>cost</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>triggerConditions#format=json</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>cost</t>
+          <t>weight</t>
         </is>
       </c>
     </row>
@@ -583,20 +582,15 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>array,array,int</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>int</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>array,array,int</t>
-        </is>
-      </c>
       <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>array,array,int</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -614,7 +608,6 @@
       <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="n"/>
       <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
@@ -629,32 +622,27 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>BUFF标题</t>
+          <t>BUFF名字</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>BUFF内容</t>
+          <t>BUFF介绍</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>TYPE</t>
+          <t>BUFF对属性的修改，格式[[属性ID,值]]</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>BUFF生效时的属性修改，格式[[属性ID,值]]</t>
+          <t>BUFF花费</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>BUFF触发条件，格式[[属性ID,阈值]]；阈值语义由运行时解释</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Cost</t>
+          <t>BUFF权重</t>
         </is>
       </c>
     </row>
@@ -670,24 +658,19 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>提高月愿望单增长，并少量追加当前愿望单。</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
+          <t>提高周愿望增长，并少量追加当前愿望单。</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>[[1004,500],[1009,1]]</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>[[1009,5]]</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="n">
+      <c r="F5" s="2" t="n">
         <v>15</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="6" ht="28.5" customHeight="1">
@@ -705,21 +688,16 @@
           <t>围绕愿望单和质量分的整数属性调整。</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>[[1009,1],[1010,2]]</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>[[1009,3],[1010,6]]</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="n">
+      <c r="F6" s="2" t="n">
         <v>25</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="7" ht="28.5" customHeight="1">
@@ -734,24 +712,19 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>同时调整月愿望单增长、画面、氛围、愿望单、质量分和Bug。</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
+          <t>同时调整周愿望增长、画面、氛围、愿望单、质量分和Bug。</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>[[1004,300],[1006,50],[1007,10],[1009,1],[1010,2],[1005,2]]</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>[[1009,4],[1010,8],[1005,12]]</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="n">
+      <c r="F7" s="2" t="n">
         <v>40</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Luban config data
</commit_message>
<xml_diff>
--- a/Config/Luban/Datas/#game.buff.xlsx
+++ b/Config/Luban/Datas/#game.buff.xlsx
@@ -1512,7 +1512,7 @@
         <v>43</v>
       </c>
       <c r="G10" s="2">
-        <v>14</v>
+        <v>40000</v>
       </c>
       <c r="H10" s="2">
         <v>125</v>
@@ -1536,7 +1536,7 @@
         <v>47</v>
       </c>
       <c r="G11" s="2">
-        <v>28</v>
+        <v>55000</v>
       </c>
       <c r="H11" s="2">
         <v>80</v>
@@ -1560,7 +1560,7 @@
         <v>51</v>
       </c>
       <c r="G12" s="2">
-        <v>30</v>
+        <v>90000</v>
       </c>
       <c r="H12" s="2">
         <v>70</v>
@@ -1584,7 +1584,7 @@
         <v>55</v>
       </c>
       <c r="G13" s="2">
-        <v>35</v>
+        <v>70000</v>
       </c>
       <c r="H13" s="2">
         <v>65</v>
@@ -1608,7 +1608,7 @@
         <v>59</v>
       </c>
       <c r="G14" s="2">
-        <v>32</v>
+        <v>65000</v>
       </c>
       <c r="H14" s="2">
         <v>75</v>
@@ -1632,7 +1632,7 @@
         <v>63</v>
       </c>
       <c r="G15" s="2">
-        <v>26</v>
+        <v>80000</v>
       </c>
       <c r="H15" s="2">
         <v>85</v>
@@ -1656,7 +1656,7 @@
         <v>67</v>
       </c>
       <c r="G16" s="2">
-        <v>40</v>
+        <v>80000</v>
       </c>
       <c r="H16" s="2">
         <v>55</v>
@@ -1680,7 +1680,7 @@
         <v>71</v>
       </c>
       <c r="G17" s="2">
-        <v>45</v>
+        <v>95000</v>
       </c>
       <c r="H17" s="2">
         <v>45</v>

</xml_diff>